<commit_message>
Configuración para despliegue en Render
</commit_message>
<xml_diff>
--- a/media/prediccion_ia_12.xlsx
+++ b/media/prediccion_ia_12.xlsx
@@ -484,23 +484,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.18</v>
+        <v>4.2</v>
       </c>
       <c r="C2" t="n">
-        <v>3.8</v>
+        <v>3.86</v>
       </c>
       <c r="D2" t="n">
-        <v>-9.1</v>
+        <v>-8.07</v>
       </c>
       <c r="E2" t="n">
-        <v>74.14</v>
+        <v>72.89</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.1041</v>
       </c>
       <c r="G2" t="n">
         <v>3.06</v>
@@ -559,1521 +559,1521 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.17</v>
+        <v>4.05</v>
       </c>
       <c r="C2" t="n">
-        <v>3.87</v>
+        <v>3.85</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2991</v>
+        <v>0.2024</v>
       </c>
       <c r="E2" t="n">
-        <v>7.172661870503597</v>
+        <v>4.997530864197531</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.15</v>
+        <v>4.1</v>
       </c>
       <c r="C3" t="n">
-        <v>3.86</v>
+        <v>3.83</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2888</v>
+        <v>0.2681</v>
       </c>
       <c r="E3" t="n">
-        <v>6.959036144578312</v>
+        <v>6.539024390243902</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="C4" t="n">
-        <v>3.85</v>
+        <v>3.82</v>
       </c>
       <c r="D4" t="n">
-        <v>0.351</v>
+        <v>0.2765</v>
       </c>
       <c r="E4" t="n">
-        <v>8.357142857142856</v>
+        <v>6.743902439024392</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.13</v>
+        <v>4.05</v>
       </c>
       <c r="C5" t="n">
-        <v>3.85</v>
+        <v>3.82</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2812</v>
+        <v>0.2332</v>
       </c>
       <c r="E5" t="n">
-        <v>6.808716707021792</v>
+        <v>5.758024691358025</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.15</v>
+        <v>4.1</v>
       </c>
       <c r="C6" t="n">
-        <v>3.84</v>
+        <v>3.8</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3086</v>
+        <v>0.3</v>
       </c>
       <c r="E6" t="n">
-        <v>7.436144578313251</v>
+        <v>7.317073170731708</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.15</v>
+        <v>4.1</v>
       </c>
       <c r="C7" t="n">
-        <v>3.84</v>
+        <v>3.79</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3093</v>
+        <v>0.3053</v>
       </c>
       <c r="E7" t="n">
-        <v>7.453012048192771</v>
+        <v>7.446341463414635</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.15</v>
+        <v>4.12</v>
       </c>
       <c r="C8" t="n">
-        <v>3.84</v>
+        <v>3.79</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3065</v>
+        <v>0.3281</v>
       </c>
       <c r="E8" t="n">
-        <v>7.385542168674698</v>
+        <v>7.963592233009709</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.05</v>
+        <v>4.1</v>
       </c>
       <c r="C9" t="n">
-        <v>3.85</v>
+        <v>3.8</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2024</v>
+        <v>0.305</v>
       </c>
       <c r="E9" t="n">
-        <v>4.997530864197531</v>
+        <v>7.439024390243904</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4.1</v>
+        <v>3.97</v>
       </c>
       <c r="C10" t="n">
-        <v>3.83</v>
+        <v>3.8</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2681</v>
+        <v>0.1737</v>
       </c>
       <c r="E10" t="n">
-        <v>6.539024390243902</v>
+        <v>4.375314861460957</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.1</v>
+        <v>3.92</v>
       </c>
       <c r="C11" t="n">
-        <v>3.82</v>
+        <v>3.78</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2765</v>
+        <v>0.1426</v>
       </c>
       <c r="E11" t="n">
-        <v>6.743902439024392</v>
+        <v>3.637755102040816</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.05</v>
+        <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>3.82</v>
+        <v>3.75</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2332</v>
+        <v>0.2542</v>
       </c>
       <c r="E12" t="n">
-        <v>5.758024691358025</v>
+        <v>6.355</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>3.8</v>
+        <v>3.74</v>
       </c>
       <c r="D13" t="n">
-        <v>0.3</v>
+        <v>0.2631</v>
       </c>
       <c r="E13" t="n">
-        <v>7.317073170731708</v>
+        <v>6.5775</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>3.79</v>
+        <v>3.73</v>
       </c>
       <c r="D14" t="n">
-        <v>0.3053</v>
+        <v>0.268</v>
       </c>
       <c r="E14" t="n">
-        <v>7.446341463414635</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4.12</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>3.79</v>
+        <v>3.73</v>
       </c>
       <c r="D15" t="n">
-        <v>0.3281</v>
+        <v>0.2694</v>
       </c>
       <c r="E15" t="n">
-        <v>7.963592233009709</v>
+        <v>6.734999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>3.8</v>
+        <v>3.73</v>
       </c>
       <c r="D16" t="n">
-        <v>0.305</v>
+        <v>0.2701</v>
       </c>
       <c r="E16" t="n">
-        <v>7.439024390243904</v>
+        <v>6.7525</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.97</v>
+        <v>4.05</v>
       </c>
       <c r="C17" t="n">
-        <v>3.8</v>
+        <v>3.73</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1737</v>
+        <v>0.3189</v>
       </c>
       <c r="E17" t="n">
-        <v>4.375314861460957</v>
+        <v>7.874074074074075</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3.92</v>
+        <v>4.1</v>
       </c>
       <c r="C18" t="n">
-        <v>3.78</v>
+        <v>3.74</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1426</v>
+        <v>0.3604</v>
       </c>
       <c r="E18" t="n">
-        <v>3.637755102040816</v>
+        <v>8.790243902439025</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>4.06</v>
       </c>
       <c r="C19" t="n">
         <v>3.75</v>
       </c>
       <c r="D19" t="n">
-        <v>0.2542</v>
+        <v>0.3078</v>
       </c>
       <c r="E19" t="n">
-        <v>6.355</v>
+        <v>7.581280788177342</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>4.14</v>
       </c>
       <c r="C20" t="n">
-        <v>3.74</v>
+        <v>3.76</v>
       </c>
       <c r="D20" t="n">
-        <v>0.2631</v>
+        <v>0.3846</v>
       </c>
       <c r="E20" t="n">
-        <v>6.5775</v>
+        <v>9.289855072463769</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>4.03</v>
       </c>
       <c r="C21" t="n">
-        <v>3.73</v>
+        <v>3.77</v>
       </c>
       <c r="D21" t="n">
-        <v>0.268</v>
+        <v>0.2612</v>
       </c>
       <c r="E21" t="n">
-        <v>6.7</v>
+        <v>6.481389578163771</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>4.08</v>
       </c>
       <c r="C22" t="n">
-        <v>3.73</v>
+        <v>3.76</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2694</v>
+        <v>0.319</v>
       </c>
       <c r="E22" t="n">
-        <v>6.734999999999999</v>
+        <v>7.818627450980392</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>4.09</v>
       </c>
       <c r="C23" t="n">
-        <v>3.73</v>
+        <v>3.76</v>
       </c>
       <c r="D23" t="n">
-        <v>0.2701</v>
+        <v>0.3295</v>
       </c>
       <c r="E23" t="n">
-        <v>6.7525</v>
+        <v>8.056234718826406</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>4.05</v>
       </c>
       <c r="C24" t="n">
-        <v>3.73</v>
+        <v>3.76</v>
       </c>
       <c r="D24" t="n">
-        <v>0.3189</v>
+        <v>0.2873</v>
       </c>
       <c r="E24" t="n">
-        <v>7.874074074074075</v>
+        <v>7.093827160493828</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4.1</v>
+        <v>4.07</v>
       </c>
       <c r="C25" t="n">
-        <v>3.74</v>
+        <v>3.76</v>
       </c>
       <c r="D25" t="n">
-        <v>0.3604</v>
+        <v>0.3068</v>
       </c>
       <c r="E25" t="n">
-        <v>8.790243902439025</v>
+        <v>7.538083538083538</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4.06</v>
+        <v>4.05</v>
       </c>
       <c r="C26" t="n">
-        <v>3.75</v>
+        <v>3.77</v>
       </c>
       <c r="D26" t="n">
-        <v>0.3078</v>
+        <v>0.2786</v>
       </c>
       <c r="E26" t="n">
-        <v>7.581280788177342</v>
+        <v>6.879012345679013</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4.14</v>
+        <v>3.96</v>
       </c>
       <c r="C27" t="n">
-        <v>3.76</v>
+        <v>3.77</v>
       </c>
       <c r="D27" t="n">
-        <v>0.3846</v>
+        <v>0.1893</v>
       </c>
       <c r="E27" t="n">
-        <v>9.289855072463769</v>
+        <v>4.78030303030303</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4.03</v>
+        <v>4</v>
       </c>
       <c r="C28" t="n">
-        <v>3.77</v>
+        <v>3.75</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2612</v>
+        <v>0.25</v>
       </c>
       <c r="E28" t="n">
-        <v>6.481389578163771</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4.08</v>
+        <v>3.9</v>
       </c>
       <c r="C29" t="n">
-        <v>3.76</v>
+        <v>3.74</v>
       </c>
       <c r="D29" t="n">
-        <v>0.319</v>
+        <v>0.1608</v>
       </c>
       <c r="E29" t="n">
-        <v>7.818627450980392</v>
+        <v>4.123076923076923</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4.09</v>
+        <v>3.96</v>
       </c>
       <c r="C30" t="n">
-        <v>3.76</v>
+        <v>3.72</v>
       </c>
       <c r="D30" t="n">
-        <v>0.3295</v>
+        <v>0.244</v>
       </c>
       <c r="E30" t="n">
-        <v>8.056234718826406</v>
+        <v>6.161616161616162</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4.05</v>
+        <v>3.93</v>
       </c>
       <c r="C31" t="n">
-        <v>3.76</v>
+        <v>3.71</v>
       </c>
       <c r="D31" t="n">
-        <v>0.2873</v>
+        <v>0.2215</v>
       </c>
       <c r="E31" t="n">
-        <v>7.093827160493828</v>
+        <v>5.636132315521628</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4.07</v>
+        <v>3.96</v>
       </c>
       <c r="C32" t="n">
-        <v>3.76</v>
+        <v>3.7</v>
       </c>
       <c r="D32" t="n">
-        <v>0.3068</v>
+        <v>0.2624</v>
       </c>
       <c r="E32" t="n">
-        <v>7.538083538083538</v>
+        <v>6.626262626262627</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4.05</v>
+        <v>3.96</v>
       </c>
       <c r="C33" t="n">
-        <v>3.77</v>
+        <v>3.69</v>
       </c>
       <c r="D33" t="n">
-        <v>0.2786</v>
+        <v>0.2669</v>
       </c>
       <c r="E33" t="n">
-        <v>6.879012345679013</v>
+        <v>6.739898989898991</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3.96</v>
+        <v>3.9</v>
       </c>
       <c r="C34" t="n">
-        <v>3.77</v>
+        <v>3.69</v>
       </c>
       <c r="D34" t="n">
-        <v>0.1893</v>
+        <v>0.2095</v>
       </c>
       <c r="E34" t="n">
-        <v>4.78030303030303</v>
+        <v>5.371794871794871</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="C35" t="n">
-        <v>3.75</v>
+        <v>3.68</v>
       </c>
       <c r="D35" t="n">
-        <v>0.25</v>
+        <v>0.2244</v>
       </c>
       <c r="E35" t="n">
-        <v>6.25</v>
+        <v>5.753846153846154</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3.9</v>
+        <v>3.85</v>
       </c>
       <c r="C36" t="n">
-        <v>3.74</v>
+        <v>3.67</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1608</v>
+        <v>0.1895</v>
       </c>
       <c r="E36" t="n">
-        <v>4.123076923076923</v>
+        <v>4.922077922077922</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3.96</v>
+        <v>3.78</v>
       </c>
       <c r="C37" t="n">
-        <v>3.72</v>
+        <v>3.65</v>
       </c>
       <c r="D37" t="n">
-        <v>0.244</v>
+        <v>0.13</v>
       </c>
       <c r="E37" t="n">
-        <v>6.161616161616162</v>
+        <v>3.43915343915344</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3.93</v>
+        <v>3.79</v>
       </c>
       <c r="C38" t="n">
-        <v>3.71</v>
+        <v>3.62</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2215</v>
+        <v>0.1663</v>
       </c>
       <c r="E38" t="n">
-        <v>5.636132315521628</v>
+        <v>4.387862796833773</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3.96</v>
+        <v>3.78</v>
       </c>
       <c r="C39" t="n">
-        <v>3.7</v>
+        <v>3.61</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2624</v>
+        <v>0.1783</v>
       </c>
       <c r="E39" t="n">
-        <v>6.626262626262627</v>
+        <v>4.716931216931217</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3.96</v>
+        <v>3.77</v>
       </c>
       <c r="C40" t="n">
-        <v>3.69</v>
+        <v>3.59</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2669</v>
+        <v>0.1817</v>
       </c>
       <c r="E40" t="n">
-        <v>6.739898989898991</v>
+        <v>4.819628647214854</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3.9</v>
+        <v>3.77</v>
       </c>
       <c r="C41" t="n">
-        <v>3.69</v>
+        <v>3.57</v>
       </c>
       <c r="D41" t="n">
-        <v>0.2095</v>
+        <v>0.1988</v>
       </c>
       <c r="E41" t="n">
-        <v>5.371794871794871</v>
+        <v>5.273209549071618</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3.9</v>
+        <v>3.77</v>
       </c>
       <c r="C42" t="n">
-        <v>3.68</v>
+        <v>3.57</v>
       </c>
       <c r="D42" t="n">
-        <v>0.2244</v>
+        <v>0.203</v>
       </c>
       <c r="E42" t="n">
-        <v>5.753846153846154</v>
+        <v>5.384615384615385</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3.85</v>
+        <v>3.75</v>
       </c>
       <c r="C43" t="n">
-        <v>3.67</v>
+        <v>3.56</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1895</v>
+        <v>0.1905</v>
       </c>
       <c r="E43" t="n">
-        <v>4.922077922077922</v>
+        <v>5.08</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3.78</v>
+        <v>3.77</v>
       </c>
       <c r="C44" t="n">
-        <v>3.65</v>
+        <v>3.55</v>
       </c>
       <c r="D44" t="n">
-        <v>0.13</v>
+        <v>0.2184</v>
       </c>
       <c r="E44" t="n">
-        <v>3.43915343915344</v>
+        <v>5.793103448275862</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3.79</v>
+        <v>3.75</v>
       </c>
       <c r="C45" t="n">
-        <v>3.62</v>
+        <v>3.54</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1663</v>
+        <v>0.2021</v>
       </c>
       <c r="E45" t="n">
-        <v>4.387862796833773</v>
+        <v>5.389333333333333</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3.78</v>
+        <v>3.74</v>
       </c>
       <c r="C46" t="n">
-        <v>3.61</v>
+        <v>3.54</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1783</v>
+        <v>0.2041</v>
       </c>
       <c r="E46" t="n">
-        <v>4.716931216931217</v>
+        <v>5.457219251336898</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3.77</v>
+        <v>3.69</v>
       </c>
       <c r="C47" t="n">
-        <v>3.59</v>
+        <v>3.52</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1817</v>
+        <v>0.1667</v>
       </c>
       <c r="E47" t="n">
-        <v>4.819628647214854</v>
+        <v>4.517615176151761</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3.77</v>
+        <v>3.75</v>
       </c>
       <c r="C48" t="n">
-        <v>3.57</v>
+        <v>3.5</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1988</v>
+        <v>0.2443</v>
       </c>
       <c r="E48" t="n">
-        <v>5.273209549071618</v>
+        <v>6.514666666666666</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3.77</v>
+        <v>3.78</v>
       </c>
       <c r="C49" t="n">
-        <v>3.57</v>
+        <v>3.51</v>
       </c>
       <c r="D49" t="n">
-        <v>0.203</v>
+        <v>0.2739</v>
       </c>
       <c r="E49" t="n">
-        <v>5.384615384615385</v>
+        <v>7.246031746031746</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3.75</v>
+        <v>3.7</v>
       </c>
       <c r="C50" t="n">
-        <v>3.56</v>
+        <v>3.52</v>
       </c>
       <c r="D50" t="n">
-        <v>0.1905</v>
+        <v>0.1799</v>
       </c>
       <c r="E50" t="n">
-        <v>5.08</v>
+        <v>4.862162162162162</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>3.77</v>
+        <v>3.74</v>
       </c>
       <c r="C51" t="n">
-        <v>3.55</v>
+        <v>3.52</v>
       </c>
       <c r="D51" t="n">
-        <v>0.2184</v>
+        <v>0.2162</v>
       </c>
       <c r="E51" t="n">
-        <v>5.793103448275862</v>
+        <v>5.780748663101605</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>3.75</v>
+        <v>3.74</v>
       </c>
       <c r="C52" t="n">
-        <v>3.54</v>
+        <v>3.53</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2021</v>
+        <v>0.2091</v>
       </c>
       <c r="E52" t="n">
-        <v>5.389333333333333</v>
+        <v>5.590909090909091</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>3.74</v>
+        <v>3.75</v>
       </c>
       <c r="C53" t="n">
         <v>3.54</v>
       </c>
       <c r="D53" t="n">
-        <v>0.2041</v>
+        <v>0.2117</v>
       </c>
       <c r="E53" t="n">
-        <v>5.457219251336898</v>
+        <v>5.645333333333333</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>3.69</v>
+        <v>3.75</v>
       </c>
       <c r="C54" t="n">
-        <v>3.52</v>
+        <v>3.54</v>
       </c>
       <c r="D54" t="n">
-        <v>0.1667</v>
+        <v>0.2032</v>
       </c>
       <c r="E54" t="n">
-        <v>4.517615176151761</v>
+        <v>5.418666666666667</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>3.75</v>
       </c>
       <c r="C55" t="n">
-        <v>3.5</v>
+        <v>3.55</v>
       </c>
       <c r="D55" t="n">
-        <v>0.2443</v>
+        <v>0.2046</v>
       </c>
       <c r="E55" t="n">
-        <v>6.514666666666666</v>
+        <v>5.456</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>3.78</v>
+        <v>3.75</v>
       </c>
       <c r="C56" t="n">
-        <v>3.51</v>
+        <v>3.55</v>
       </c>
       <c r="D56" t="n">
-        <v>0.2739</v>
+        <v>0.2041</v>
       </c>
       <c r="E56" t="n">
-        <v>7.246031746031746</v>
+        <v>5.442666666666667</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>3.7</v>
+        <v>3.74</v>
       </c>
       <c r="C57" t="n">
-        <v>3.52</v>
+        <v>3.54</v>
       </c>
       <c r="D57" t="n">
-        <v>0.1799</v>
+        <v>0.1976</v>
       </c>
       <c r="E57" t="n">
-        <v>4.862162162162162</v>
+        <v>5.283422459893048</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3.74</v>
+        <v>3.7</v>
       </c>
       <c r="C58" t="n">
-        <v>3.52</v>
+        <v>3.54</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2162</v>
+        <v>0.1635</v>
       </c>
       <c r="E58" t="n">
-        <v>5.780748663101605</v>
+        <v>4.418918918918919</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>3.74</v>
+        <v>3.68</v>
       </c>
       <c r="C59" t="n">
-        <v>3.53</v>
+        <v>3.52</v>
       </c>
       <c r="D59" t="n">
-        <v>0.2091</v>
+        <v>0.1577</v>
       </c>
       <c r="E59" t="n">
-        <v>5.590909090909091</v>
+        <v>4.285326086956522</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>3.75</v>
+        <v>3.7</v>
       </c>
       <c r="C60" t="n">
-        <v>3.54</v>
+        <v>3.51</v>
       </c>
       <c r="D60" t="n">
-        <v>0.2117</v>
+        <v>0.1959</v>
       </c>
       <c r="E60" t="n">
-        <v>5.645333333333333</v>
+        <v>5.294594594594594</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>3.75</v>
+        <v>3.66</v>
       </c>
       <c r="C61" t="n">
-        <v>3.54</v>
+        <v>3.5</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2032</v>
+        <v>0.1613</v>
       </c>
       <c r="E61" t="n">
-        <v>5.418666666666667</v>
+        <v>4.407103825136612</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>3.75</v>
+        <v>3.67</v>
       </c>
       <c r="C62" t="n">
-        <v>3.55</v>
+        <v>3.48</v>
       </c>
       <c r="D62" t="n">
-        <v>0.2046</v>
+        <v>0.1843</v>
       </c>
       <c r="E62" t="n">
-        <v>5.456</v>
+        <v>5.021798365122616</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>3.75</v>
+        <v>3.55</v>
       </c>
       <c r="C63" t="n">
-        <v>3.55</v>
+        <v>3.47</v>
       </c>
       <c r="D63" t="n">
-        <v>0.2041</v>
+        <v>0.07870000000000001</v>
       </c>
       <c r="E63" t="n">
-        <v>5.442666666666667</v>
+        <v>2.216901408450704</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>3.74</v>
+        <v>3.6</v>
       </c>
       <c r="C64" t="n">
-        <v>3.54</v>
+        <v>3.44</v>
       </c>
       <c r="D64" t="n">
-        <v>0.1976</v>
+        <v>0.1644</v>
       </c>
       <c r="E64" t="n">
-        <v>5.283422459893048</v>
+        <v>4.566666666666666</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>3.7</v>
+        <v>3.97</v>
       </c>
       <c r="C65" t="n">
-        <v>3.54</v>
+        <v>3.42</v>
       </c>
       <c r="D65" t="n">
-        <v>0.1635</v>
+        <v>0.5523</v>
       </c>
       <c r="E65" t="n">
-        <v>4.418918918918919</v>
+        <v>13.91183879093199</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>3.68</v>
+        <v>3.93</v>
       </c>
       <c r="C66" t="n">
-        <v>3.52</v>
+        <v>3.49</v>
       </c>
       <c r="D66" t="n">
-        <v>0.1577</v>
+        <v>0.4396</v>
       </c>
       <c r="E66" t="n">
-        <v>4.285326086956522</v>
+        <v>11.18575063613232</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>3.7</v>
+        <v>4.02</v>
       </c>
       <c r="C67" t="n">
-        <v>3.51</v>
+        <v>3.55</v>
       </c>
       <c r="D67" t="n">
-        <v>0.1959</v>
+        <v>0.4738</v>
       </c>
       <c r="E67" t="n">
-        <v>5.294594594594594</v>
+        <v>11.7860696517413</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>3.66</v>
+        <v>4.07</v>
       </c>
       <c r="C68" t="n">
-        <v>3.5</v>
+        <v>3.61</v>
       </c>
       <c r="D68" t="n">
-        <v>0.1613</v>
+        <v>0.4617</v>
       </c>
       <c r="E68" t="n">
-        <v>4.407103825136612</v>
+        <v>11.34398034398034</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>3.67</v>
+        <v>4.07</v>
       </c>
       <c r="C69" t="n">
-        <v>3.48</v>
+        <v>3.66</v>
       </c>
       <c r="D69" t="n">
-        <v>0.1843</v>
+        <v>0.4105</v>
       </c>
       <c r="E69" t="n">
-        <v>5.021798365122616</v>
+        <v>10.08599508599509</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>3.55</v>
+        <v>4.09</v>
       </c>
       <c r="C70" t="n">
-        <v>3.47</v>
+        <v>3.7</v>
       </c>
       <c r="D70" t="n">
-        <v>0.07870000000000001</v>
+        <v>0.3925</v>
       </c>
       <c r="E70" t="n">
-        <v>2.216901408450704</v>
+        <v>9.596577017114916</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>3.6</v>
+        <v>4.07</v>
       </c>
       <c r="C71" t="n">
-        <v>3.44</v>
+        <v>3.73</v>
       </c>
       <c r="D71" t="n">
-        <v>0.1644</v>
+        <v>0.3382</v>
       </c>
       <c r="E71" t="n">
-        <v>4.566666666666666</v>
+        <v>8.309582309582309</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>3.97</v>
+        <v>4.09</v>
       </c>
       <c r="C72" t="n">
-        <v>3.42</v>
+        <v>3.75</v>
       </c>
       <c r="D72" t="n">
-        <v>0.5523</v>
+        <v>0.3387</v>
       </c>
       <c r="E72" t="n">
-        <v>13.91183879093199</v>
+        <v>8.28117359413203</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>3.93</v>
+        <v>4.06</v>
       </c>
       <c r="C73" t="n">
-        <v>3.49</v>
+        <v>3.77</v>
       </c>
       <c r="D73" t="n">
-        <v>0.4396</v>
+        <v>0.2927</v>
       </c>
       <c r="E73" t="n">
-        <v>11.18575063613232</v>
+        <v>7.209359605911331</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>4.02</v>
+        <v>4.18</v>
       </c>
       <c r="C74" t="n">
-        <v>3.55</v>
+        <v>3.78</v>
       </c>
       <c r="D74" t="n">
-        <v>0.4738</v>
+        <v>0.4031</v>
       </c>
       <c r="E74" t="n">
-        <v>11.7860696517413</v>
+        <v>9.64354066985646</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4.07</v>
+        <v>4.13</v>
       </c>
       <c r="C75" t="n">
-        <v>3.61</v>
+        <v>3.8</v>
       </c>
       <c r="D75" t="n">
-        <v>0.4617</v>
+        <v>0.3293</v>
       </c>
       <c r="E75" t="n">
-        <v>11.34398034398034</v>
+        <v>7.973365617433414</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4.07</v>
+        <v>4.18</v>
       </c>
       <c r="C76" t="n">
-        <v>3.66</v>
+        <v>3.81</v>
       </c>
       <c r="D76" t="n">
-        <v>0.4105</v>
+        <v>0.3696</v>
       </c>
       <c r="E76" t="n">
-        <v>10.08599508599509</v>
+        <v>8.842105263157896</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>4.09</v>
+        <v>4.18</v>
       </c>
       <c r="C77" t="n">
-        <v>3.7</v>
+        <v>3.82</v>
       </c>
       <c r="D77" t="n">
-        <v>0.3925</v>
+        <v>0.3577</v>
       </c>
       <c r="E77" t="n">
-        <v>9.596577017114916</v>
+        <v>8.557416267942584</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>4.07</v>
+        <v>4.19</v>
       </c>
       <c r="C78" t="n">
-        <v>3.73</v>
+        <v>3.84</v>
       </c>
       <c r="D78" t="n">
-        <v>0.3382</v>
+        <v>0.3525</v>
       </c>
       <c r="E78" t="n">
-        <v>8.309582309582309</v>
+        <v>8.41288782816229</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>4.09</v>
+        <v>4.19</v>
       </c>
       <c r="C79" t="n">
-        <v>3.75</v>
+        <v>3.85</v>
       </c>
       <c r="D79" t="n">
-        <v>0.3387</v>
+        <v>0.3386</v>
       </c>
       <c r="E79" t="n">
-        <v>8.28117359413203</v>
+        <v>8.081145584725537</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>4.06</v>
+        <v>4.2</v>
       </c>
       <c r="C80" t="n">
-        <v>3.77</v>
+        <v>3.85</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2927</v>
+        <v>0.3442</v>
       </c>
       <c r="E80" t="n">
-        <v>7.209359605911331</v>
+        <v>8.195238095238096</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>4.18</v>
+        <v>4.2</v>
       </c>
       <c r="C81" t="n">
-        <v>3.78</v>
+        <v>3.86</v>
       </c>
       <c r="D81" t="n">
-        <v>0.4031</v>
+        <v>0.343</v>
       </c>
       <c r="E81" t="n">
-        <v>9.64354066985646</v>
+        <v>8.166666666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>